<commit_message>
feat(sf2): daily attendance report of learners file export
</commit_message>
<xml_diff>
--- a/backend/services/forms/output_data/SF1_506_filled.xlsx
+++ b/backend/services/forms/output_data/SF1_506_filled.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="32">
+  <fonts count="33">
     <font>
       <name val="Arial"/>
       <charset val="134"/>
@@ -95,6 +95,14 @@
       <charset val="134"/>
       <color theme="1"/>
       <sz val="6"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -738,31 +746,28 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="12" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="43" fontId="13" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="12" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="44" fontId="13" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="12" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="9" fontId="13" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="12" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="41" fontId="13" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="12" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="42" fontId="13" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="18" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="18" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1">
@@ -771,115 +776,118 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="19" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="19" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="20" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="19" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="20" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="21" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="22" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="21" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="21" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="22" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="23" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="21" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="24" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="23" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="25" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="24" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="6" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="25" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="7" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="6" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="8" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="7" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="9" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="8" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="10" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="9" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="11" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="10" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="12" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="11" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="13" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="12" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="14" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="13" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="15" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="14" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="16" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="15" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="17" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="16" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="18" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="17" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="19" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="18" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="20" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="19" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="21" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="20" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="22" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="21" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="23" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="22" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="24" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="23" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="25" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="24" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="26" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="25" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="27" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="26" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="28" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="27" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="29" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="28" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="30" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="29" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="31" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="30" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="32" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="32" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -983,16 +991,14 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -7904,7 +7910,11 @@
           <t>JOHN CRUZ</t>
         </is>
       </c>
-      <c r="AN71" s="39" t="n"/>
+      <c r="AN71" s="39" t="inlineStr">
+        <is>
+          <t>LOURDES ABELLA MONTEFRIO</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="12.75" customHeight="1">
       <c r="A72" s="66" t="n"/>
@@ -7955,7 +7965,7 @@
       <c r="AI73" s="69" t="n"/>
       <c r="AJ73" s="69" t="n"/>
       <c r="AK73" s="69" t="n"/>
-      <c r="AN73" s="44" t="inlineStr">
+      <c r="AN73" s="39" t="inlineStr">
         <is>
           <t>(Signature of School Head over Printed Name)</t>
         </is>
@@ -7985,7 +7995,7 @@
       <c r="Z74" s="53" t="n"/>
       <c r="AA74" s="19" t="inlineStr"/>
       <c r="AB74" s="53" t="n"/>
-      <c r="AE74" s="44" t="inlineStr">
+      <c r="AE74" s="39" t="inlineStr">
         <is>
           <t>(Signature of Adviser over Printed Name)</t>
         </is>

</xml_diff>